<commit_message>
chore(swiss): checkpoint v23 docs and generated artifacts
</commit_message>
<xml_diff>
--- a/research/yjs-manual-opt/swiss/products/v23/i18n/workbooks/de.xlsx
+++ b/research/yjs-manual-opt/swiss/products/v23/i18n/workbooks/de.xlsx
@@ -4625,7 +4625,7 @@
         <v>**真空密封后袋子漏气**</v>
       </c>
       <c r="E184" t="str">
-        <v>**真空密封后袋子漏气**</v>
+        <v>**Beutel undicht nach dem Vakuumieren**</v>
       </c>
       <c r="F184" t="str">
         <v>review</v>
@@ -4648,7 +4648,7 @@
         <v>高温胶布破损或脱落</v>
       </c>
       <c r="E185" t="str">
-        <v>高温胶布破损或脱落</v>
+        <v>Das Hochtemperaturband ist beschädigt oder hat sich gelöst</v>
       </c>
       <c r="F185" t="str">
         <v>review</v>
@@ -4671,7 +4671,7 @@
         <v>及时替换高温胶布。</v>
       </c>
       <c r="E186" t="str">
-        <v>及时替换高温胶布。</v>
+        <v>Das Hochtemperaturband rechtzeitig ersetzen.</v>
       </c>
       <c r="F186" t="str">
         <v>review</v>
@@ -4694,7 +4694,7 @@
         <v>发热温度异常导致袋子融化或密封不充分</v>
       </c>
       <c r="E187" t="str">
-        <v>发热温度异常导致袋子融化或密封不充分</v>
+        <v>Ungewöhnliche Heiztemperatur schmilzt den Beutel oder führt zu einer unzureichenden Naht</v>
       </c>
       <c r="F187" t="str">
         <v>review</v>
@@ -4717,7 +4717,7 @@
         <v>参考抽气不干净和不能密封的解决方案。</v>
       </c>
       <c r="E188" t="str">
-        <v>参考抽气不干净和不能密封的解决方案。</v>
+        <v>Siehe Lösungen für schwaches Vakuum oder unzureichende Versiegelung.</v>
       </c>
       <c r="F188" t="str">
         <v>review</v>
@@ -4740,7 +4740,7 @@
         <v>锋利物品刺穿袋子</v>
       </c>
       <c r="E189" t="str">
-        <v>锋利物品刺穿袋子</v>
+        <v>Scharfe Gegenstände durchstechen den Beutel</v>
       </c>
       <c r="F189" t="str">
         <v>review</v>
@@ -4763,7 +4763,7 @@
         <v>用纸巾或防刺穿片包裹锋利边缘，使用新袋重试。</v>
       </c>
       <c r="E190" t="str">
-        <v>用纸巾或防刺穿片包裹锋利边缘，使用新袋重试。</v>
+        <v>Scharfe Kanten mit Küchenpapier oder Schutzlage umwickeln und mit einem neuen Beutel erneut versuchen.</v>
       </c>
       <c r="F190" t="str">
         <v>review</v>
@@ -5177,7 +5177,7 @@
         <v>一些水果和蔬菜在包装前如果没有正确地焯熟，或者热的食物，会释放气体，导致真空袋没有收紧，此类情况属于正常表现，不属于漏气。</v>
       </c>
       <c r="E208" t="str">
-        <v>一些水果和蔬菜在包装前如果没有正确地焯熟，或者热的食物，会释放气体，导致真空袋没有收紧，此类情况属于正常表现，不属于漏气。</v>
+        <v>Einige Obst- und Gemüsesorten können Gas abgeben, wenn sie vor dem Verpacken nicht richtig blanchiert wurden. Auch heiße Lebensmittel können Gas abgeben. Wenn sich der Beutel in diesen Fällen nicht straff zusammenzieht, ist das normal und kein Leck.</v>
       </c>
       <c r="F208" t="str">
         <v>review</v>
@@ -5200,7 +5200,7 @@
         <v>提示</v>
       </c>
       <c r="E209" t="str">
-        <v>提示</v>
+        <v>Hinweis</v>
       </c>
       <c r="F209" t="str">
         <v>review</v>
@@ -5223,7 +5223,7 @@
         <v>若以上故障排除方案均无法解决问题，请联系客服指引解决，请不要擅自拆卸机器。</v>
       </c>
       <c r="E210" t="str">
-        <v>若以上故障排除方案均无法解决问题，请联系客服指引解决，请不要擅自拆卸机器。</v>
+        <v>Wenn das Problem nach den obigen Schritten weiterhin besteht, wenden Sie sich an den Kundendienst. Zerlegen Sie das Gerät nicht selbst.</v>
       </c>
       <c r="F210" t="str">
         <v>review</v>
@@ -5499,7 +5499,7 @@
         <v>**错误报警（蜂鸣声长鸣 + 指示灯快闪）**</v>
       </c>
       <c r="E222" t="str">
-        <v>**错误报警（蜂鸣声长鸣 + 指示灯快闪）**</v>
+        <v>**Fehleralarm (langer Signalton + schnell blinkende Anzeige)**</v>
       </c>
       <c r="F222" t="str">
         <v>review</v>
@@ -5522,7 +5522,7 @@
         <v>按下 Vac&amp;Seal/Start 或 Seal 后报警</v>
       </c>
       <c r="E223" t="str">
-        <v>按下 Vac&amp;Seal/Start 或 Seal 后报警</v>
+        <v>Alarm nach Drücken von Vac&amp;Seal/Start oder Seal</v>
       </c>
       <c r="F223" t="str">
         <v>review</v>
@@ -5545,7 +5545,7 @@
         <v>检查面盖是否闭合，把手是否已下压锁紧。</v>
       </c>
       <c r="E224" t="str">
-        <v>检查面盖是否闭合，把手是否已下压锁紧。</v>
+        <v>Prüfen Sie, ob der Deckel geschlossen ist und der Griff nach unten gedrückt und verriegelt wurde.</v>
       </c>
       <c r="F224" t="str">
         <v>review</v>
@@ -5568,7 +5568,7 @@
         <v>真空工作过程中连续蜂鸣</v>
       </c>
       <c r="E225" t="str">
-        <v>真空工作过程中连续蜂鸣</v>
+        <v>Durchgehender Signalton während des Vakuumierens</v>
       </c>
       <c r="F225" t="str">
         <v>review</v>
@@ -5591,7 +5591,7 @@
         <v>机器无法达到目标压力，检查把手锁紧及袋子是否破损，更换新袋重试。</v>
       </c>
       <c r="E226" t="str">
-        <v>机器无法达到目标压力，检查把手锁紧及袋子是否破损，更换新袋重试。</v>
+        <v>Das Gerät erreicht den Zieldruck nicht. Prüfen Sie, ob der Griff verriegelt ist und der Beutel unbeschädigt ist. Mit einem neuen Beutel erneut versuchen.</v>
       </c>
       <c r="F226" t="str">
         <v>review</v>
@@ -5637,7 +5637,7 @@
         <v>如因特殊原因，导致液体进入机器内部的处理方案</v>
       </c>
       <c r="E228" t="str">
-        <v>如因特殊原因，导致液体进入机器内部的处理方案</v>
+        <v>Vorgehensweise, wenn aus besonderen Gründen Flüssigkeit in das Gerät gelangt</v>
       </c>
       <c r="F228" t="str">
         <v>review</v>
@@ -5660,7 +5660,7 @@
         <v>**液体进入真空腔中：**</v>
       </c>
       <c r="E229" t="str">
-        <v>**液体进入真空腔中：**</v>
+        <v>**Flüssigkeit gelangt in die Vakuumkammer:**</v>
       </c>
       <c r="F229" t="str">
         <v>review</v>
@@ -5683,7 +5683,7 @@
         <v>立即关闭电源，等待至少 5 分钟，让机器发热器冷却。</v>
       </c>
       <c r="E230" t="str">
-        <v>立即关闭电源，等待至少 5 分钟，让机器发热器冷却。</v>
+        <v>Gerät sofort ausschalten und mindestens 5 Minuten warten, bis der Heizer abgekühlt ist.</v>
       </c>
       <c r="F230" t="str">
         <v>review</v>
@@ -5706,7 +5706,7 @@
         <v>将液体槽取出，并清理擦干液体。</v>
       </c>
       <c r="E231" t="str">
-        <v>将液体槽取出，并清理擦干液体。</v>
+        <v>Flüssigkeitsschale herausnehmen und die Flüssigkeit aufwischen.</v>
       </c>
       <c r="F231" t="str">
         <v>review</v>
@@ -5729,7 +5729,7 @@
         <v>将真空腔中的液体擦干。</v>
       </c>
       <c r="E232" t="str">
-        <v>将真空腔中的液体擦干。</v>
+        <v>Die Flüssigkeit aus der Vakuumkammer auswischen.</v>
       </c>
       <c r="F232" t="str">
         <v>review</v>
@@ -5752,7 +5752,7 @@
         <v>将机器底部铺垫厨房纸或托盘，重新通电。</v>
       </c>
       <c r="E233" t="str">
-        <v>将机器底部铺垫厨房纸或托盘，重新通电。</v>
+        <v>Küchenpapier oder eine Auffangschale unter das Gerät legen und es wieder einschalten.</v>
       </c>
       <c r="F233" t="str">
         <v>review</v>
@@ -5775,7 +5775,7 @@
         <v>合上面盖，长按 [btn:Pulse Vac] 按键抽气 20 秒，然后点击 [btn:Stop] 排气，重复 5 次，让内部管道的液体排出。</v>
       </c>
       <c r="E234" t="str">
-        <v>合上面盖，长按 [btn:Pulse Vac] 按键抽气 20 秒，然后点击 [btn:Stop] 排气，重复 5 次，让内部管道的液体排出。</v>
+        <v>Deckel schließen, [btn:Pulse Vac] 20 Sekunden lang gedrückt halten und dann [btn:Stop] drücken, um zu entlüften. Fünfmal wiederholen, damit die Flüssigkeit aus den internen Leitungen austritt.</v>
       </c>
       <c r="F234" t="str">
         <v>review</v>
@@ -5798,7 +5798,7 @@
         <v>打开面盖，在机器底部铺垫厨房纸或托盘，将机器放置于通风处晾干 48 小时，期间不要翻倒机器。</v>
       </c>
       <c r="E235" t="str">
-        <v>打开面盖，在机器底部铺垫厨房纸或托盘，将机器放置于通风处晾干 48 小时，期间不要翻倒机器。</v>
+        <v>Deckel öffnen, Küchenpapier oder eine Auffangschale unter das Gerät legen und es 48 Stunden an einem gut belüfteten Ort trocknen lassen. Das Gerät dabei nicht kippen oder umdrehen.</v>
       </c>
       <c r="F235" t="str">
         <v>review</v>
@@ -5821,7 +5821,7 @@
         <v>**液体进入发热器：**</v>
       </c>
       <c r="E236" t="str">
-        <v>**液体进入发热器：**</v>
+        <v>**Flüssigkeit gelangt in den Heizer:**</v>
       </c>
       <c r="F236" t="str">
         <v>review</v>
@@ -5844,7 +5844,7 @@
         <v>请勿翻倒机器，关闭电源，等待 10 分钟，让发热器冷却及内部液体排出。</v>
       </c>
       <c r="E237" t="str">
-        <v>请勿翻倒机器，关闭电源，等待 10 分钟，让发热器冷却及内部液体排出。</v>
+        <v>Das Gerät nicht umdrehen. Ausschalten und 10 Minuten warten, bis der Heizer abgekühlt ist und die Flüssigkeit im Inneren ablaufen kann.</v>
       </c>
       <c r="F237" t="str">
         <v>review</v>
@@ -5867,7 +5867,7 @@
         <v>清理和擦干机器接水盘、真空腔、底部的液体。</v>
       </c>
       <c r="E238" t="str">
-        <v>清理和擦干机器接水盘、真空腔、底部的液体。</v>
+        <v>Auffangschale, Vakuumkammer und die Flüssigkeit am Geräteboden reinigen und trocknen.</v>
       </c>
       <c r="F238" t="str">
         <v>review</v>
@@ -5890,7 +5890,7 @@
         <v>打开面盖，在机器底部铺垫厨房纸或托盘，将机器放置于通风处晾干 24 小时，期间不要翻倒机器。</v>
       </c>
       <c r="E239" t="str">
-        <v>打开面盖，在机器底部铺垫厨房纸或托盘，将机器放置于通风处晾干 24 小时，期间不要翻倒机器。</v>
+        <v>Deckel öffnen, Küchenpapier oder eine Auffangschale unter das Gerät legen und es 24 Stunden an einem gut belüfteten Ort trocknen lassen. Das Gerät dabei nicht kippen oder umdrehen.</v>
       </c>
       <c r="F239" t="str">
         <v>review</v>
@@ -5913,7 +5913,7 @@
         <v>将机器底部铺垫厨房纸或托盘，重新通电。</v>
       </c>
       <c r="E240" t="str">
-        <v>将机器底部铺垫厨房纸或托盘，重新通电。</v>
+        <v>Küchenpapier oder eine Auffangschale unter das Gerät legen und es wieder einschalten.</v>
       </c>
       <c r="F240" t="str">
         <v>review</v>
@@ -5936,7 +5936,7 @@
         <v>合上面盖，长按 [btn:Pulse Vac] 按键抽气 20 秒，然后点击 [btn:Stop] 排气，重复 5 次，让内部管道的液体排出。</v>
       </c>
       <c r="E241" t="str">
-        <v>合上面盖，长按 [btn:Pulse Vac] 按键抽气 20 秒，然后点击 [btn:Stop] 排气，重复 5 次，让内部管道的液体排出。</v>
+        <v>Deckel schließen, [btn:Pulse Vac] 20 Sekunden lang gedrückt halten und dann [btn:Stop] drücken, um zu entlüften. Fünfmal wiederholen, damit die Flüssigkeit aus den internen Leitungen austritt.</v>
       </c>
       <c r="F241" t="str">
         <v>review</v>
@@ -5959,7 +5959,7 @@
         <v>打开面盖，在机器底部铺垫厨房纸或托盘，将机器放置于通风处晾干 48 小时，期间不要翻倒机器。</v>
       </c>
       <c r="E242" t="str">
-        <v>打开面盖，在机器底部铺垫厨房纸或托盘，将机器放置于通风处晾干 48 小时，期间不要翻倒机器。</v>
+        <v>Deckel öffnen, Küchenpapier oder eine Auffangschale unter das Gerät legen und es 48 Stunden an einem gut belüfteten Ort trocknen lassen. Das Gerät dabei nicht kippen oder umdrehen.</v>
       </c>
       <c r="F242" t="str">
         <v>review</v>
@@ -5982,7 +5982,7 @@
         <v>如果长期不清洁，内部管道可能会堵塞，影响抽气性能，此时请联系售后进行管道更换。</v>
       </c>
       <c r="E243" t="str">
-        <v>如果长期不清洁，内部管道可能会堵塞，影响抽气性能，此时请联系售后进行管道更换。</v>
+        <v>Werden die internen Leitungen lange nicht gereinigt, können sie verstopfen und die Saugleistung beeinträchtigen. Wenden Sie sich für einen Leitungstausch an den Kundendienst.</v>
       </c>
       <c r="F243" t="str">
         <v>review</v>
@@ -6005,7 +6005,7 @@
         <v>注意</v>
       </c>
       <c r="E244" t="str">
-        <v>注意</v>
+        <v>Achtung</v>
       </c>
       <c r="F244" t="str">
         <v>review</v>

</xml_diff>